<commit_message>
Latest Commit after xml files
</commit_message>
<xml_diff>
--- a/GroceryApplicationProject/src/test/resources/TestData.xlsx
+++ b/GroceryApplicationProject/src/test/resources/TestData.xlsx
@@ -5,15 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jaya Saketh\eclipse-workspace\GroceryApplicationProject\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jaya Saketh\git\MainProject_Obsqura\GroceryApplicationProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB8A513-D183-4A86-A62E-0726AF86D78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F22D61-86D0-4B87-A9DE-03A01C7FF5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1164" yWindow="2616" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4848" yWindow="2124" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
+    <sheet name="ManageNewsPage" sheetId="2" r:id="rId1"/>
+    <sheet name="LoginPage" sheetId="1" r:id="rId2"/>
+    <sheet name="AdminUsersPage" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>Jaya News</t>
+  </si>
   <si>
     <t>standard_user</t>
   </si>
@@ -39,25 +47,20 @@
     <t>standard_use</t>
   </si>
   <si>
-    <t>admin</t>
+    <t>AdminJaya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -86,10 +89,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -369,54 +371,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B863AB9-CB4D-4186-8371-ABC269D21BCE}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75F67B29-E8BA-4F55-8931-E54928DCC6BB}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>